<commit_message>
baselines: trim text the paired PDFs never render
Exports and hand-made baselines carried paragraphs the PDF layout omits
(Qualys Threat tails, Nessus plugin-output truncations), capping every
extractor below 1.0 on content it never saw. tools/trim_baselines.py pairs
rows to segmented blocks by name and drops paragraphs under 0.80 token
containment; 1487 paragraphs removed across 11 of 24 reports (ZAP untouched,
XML matches the PDF).
</commit_message>
<xml_diff>
--- a/resources/acunetix/Acunetix_testphp.xlsx
+++ b/resources/acunetix/Acunetix_testphp.xlsx
@@ -2016,17 +2016,7 @@
 attacks, which ensures that their content is not embedded into other pages or frames.</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Sending the proper X-Frame-Options in HTTP response headers that instruct the browser to not allow framing from other
-domains.
-X-Frame-Options: DENY  It completely denies to be loaded in frame/iframe.
-X-Frame-Options: SAMEORIGIN It allows only if the site which wants to load has a same origin.
-X-Frame-Options: ALLOW-FROM URL It grants a specific URL to load itself in a iframe. However please pay
-attention to that, not all browsers support this.
-Employing defensive code in the UI to ensure that the current frame is the most top level window.</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Clickjacking is when an attacker uses multiple transparent or opaque layers to trick a user into clicking on a button or link on

</xml_diff>